<commit_message>
análise temporal - OCO2 vc OCO2+OCO3
</commit_message>
<xml_diff>
--- a/output/estat-desc.xlsx
+++ b/output/estat-desc.xlsx
@@ -660,10 +660,10 @@
         <v>1.288654587149141</v>
       </c>
       <c r="F12">
-        <v>-0.05206752591573936</v>
+        <v>-0.05206752591573937</v>
       </c>
       <c r="G12">
-        <v>1.215106955521996</v>
+        <v>1.215106955521994</v>
       </c>
     </row>
     <row r="13">
@@ -735,7 +735,7 @@
         <v>1.380193498480505</v>
       </c>
       <c r="F15">
-        <v>0.03167685863357666</v>
+        <v>0.03167685863357665</v>
       </c>
       <c r="G15">
         <v>0.9485535811913093</v>
@@ -910,7 +910,7 @@
         <v>1.579544232783316</v>
       </c>
       <c r="F22">
-        <v>0.454634025798357</v>
+        <v>0.4546340257983569</v>
       </c>
       <c r="G22">
         <v>1.080988588732997</v>
@@ -1060,7 +1060,7 @@
         <v>1.351686916102079</v>
       </c>
       <c r="F28">
-        <v>0.007259319748710852</v>
+        <v>0.007259319748710854</v>
       </c>
       <c r="G28">
         <v>5.575260058420453</v>
@@ -1110,7 +1110,7 @@
         <v>1.120683506898008</v>
       </c>
       <c r="F30">
-        <v>-0.4178722419530688</v>
+        <v>-0.417872241953069</v>
       </c>
       <c r="G30">
         <v>1.810055065630911</v>

</xml_diff>